<commit_message>
Fix current AOFM data routes
</commit_message>
<xml_diff>
--- a/tests/testthat/fixtures/slf.xlsx
+++ b/tests/testthat/fixtures/slf.xlsx
@@ -7,8 +7,8 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Transactions" sheetId="1" r:id="rId1"/>
-    <sheet name="Notes" sheetId="2" r:id="rId2"/>
+    <sheet name="Notes" sheetId="1" r:id="rId1"/>
+    <sheet name="Transactions" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -341,94 +341,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Synthetic securities lending transactions</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Start Date</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>End Date</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Security Maturity Date</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>46174</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>46181</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>49481</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>TB 2035</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>46204</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>46211</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>49481</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>TB 2035</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>30</t>
+          <t>Synthetic SLF notes</t>
         </is>
       </c>
     </row>
@@ -439,13 +358,94 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Synthetic SLF notes</t>
+          <t>Synthetic securities lending transactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>End Date</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Security Maturity Date</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>46174</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>46181</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>49481</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>TB 2035</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>46204</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>46211</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>49481</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>TB 2035</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>30</t>
         </is>
       </c>
     </row>

</xml_diff>